<commit_message>
format pdf outfile to A4; add secont table
</commit_message>
<xml_diff>
--- a/files/results.xlsx
+++ b/files/results.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Дима документы\Python\orca_socme_processing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Дима документы\Python\orca_socme_processing\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" firstSheet="13" activeTab="27"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" firstSheet="13" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="1" r:id="rId1"/>
@@ -3275,31 +3275,31 @@
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="5">
         <v>0.39257886780000018</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="5">
         <v>0.45086568659999982</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="5">
         <v>0.2277594179999998</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="5">
         <v>0.53119373939999992</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="5">
         <v>0.51383286619999957</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="5">
         <v>0.67718290040000051</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="5">
         <v>1.5401652400000019E-2</v>
       </c>
-      <c r="J5" s="3">
+      <c r="J5" s="5">
         <v>0.24370529839999969</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="5">
         <v>0.31801963179999992</v>
       </c>
       <c r="M5">
@@ -3347,31 +3347,31 @@
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="5">
         <v>0.61293678500000048</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="5">
         <v>0.55611938179999987</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="5">
         <v>0.38272834100000003</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="5">
         <v>0.65046130559999993</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="5">
         <v>0.58942613539999966</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="5">
         <v>0.68159114720000025</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="5">
         <v>3.074888200000014E-2</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="5">
         <v>0.32395171699999992</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="5">
         <v>0.16653376799999989</v>
       </c>
       <c r="M6">
@@ -3419,31 +3419,31 @@
       <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="5">
         <v>0.34392488460000031</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="5">
         <v>0.2118951718000002</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="5">
         <v>5.5484044600000448E-2</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="5">
         <v>0.39032032160000002</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="5">
         <v>0.25390957340000009</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="5">
         <v>0.44330091740000022</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="5">
         <v>4.571515199999876E-3</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="5">
         <v>9.3307890599999777E-2</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="5">
         <v>7.0749640000000724E-4</v>
       </c>
       <c r="M7">
@@ -3491,31 +3491,31 @@
       <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="5">
         <v>0.43059319359999998</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="5">
         <v>0.25943348760000001</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="5">
         <v>0.10881838859999959</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="5">
         <v>0.43851171099999992</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="5">
         <v>0.30721670599999967</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="5">
         <v>0.51356075220000008</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="5">
         <v>9.5239899999999267E-3</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J8" s="5">
         <v>0.15317297060000001</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8" s="5">
         <v>1.496626999999862E-3</v>
       </c>
       <c r="M8">
@@ -3563,31 +3563,31 @@
       <c r="B9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="5">
         <v>3.7143561000000158E-2</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="5">
         <v>0.17469718800000009</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="5">
         <v>5.4422800000031302E-4</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="5">
         <v>0.15001644820000021</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="5">
         <v>0.26623633760000009</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="5">
         <v>0.32776131300000028</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="5">
         <v>5.4422799999898068E-5</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="5">
         <v>4.6259380000002182E-4</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="5">
         <v>4.2939589200000412E-2</v>
       </c>
       <c r="M9">
@@ -3635,31 +3635,31 @@
       <c r="B10" s="1">
         <v>6</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="5">
         <v>9.4369135199999565E-2</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="5">
         <v>0.14582589260000001</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="5">
         <v>1.8775866000000361E-3</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="5">
         <v>0.18824846519999999</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="5">
         <v>0.2121400744000006</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="5">
         <v>0.28890343380000028</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="5">
         <v>2.7211399999949041E-5</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="5">
         <v>5.4422800000031302E-4</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="5">
         <v>2.7211399999949041E-5</v>
       </c>
       <c r="M10">
@@ -3707,31 +3707,31 @@
       <c r="B11" s="1">
         <v>7</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="5">
         <v>5.9348063399999873E-2</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="5">
         <v>5.5565678799999851E-2</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="5">
         <v>1.1700902000000291E-3</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="5">
         <v>0.1069952248000003</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="5">
         <v>9.2518760000000366E-2</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="5">
         <v>0.17954081719999951</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="5">
         <v>5.4422800000342157E-5</v>
       </c>
-      <c r="J11" s="3">
+      <c r="J11" s="5">
         <v>2.9932540000032759E-4</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="5">
         <v>2.721140000039313E-5</v>
       </c>
       <c r="M11">
@@ -3779,31 +3779,31 @@
       <c r="B12" s="1">
         <v>8</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="5">
         <v>0.6111136211999999</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="5">
         <v>0.58773902859999971</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="5">
         <v>0.35165292220000038</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="5">
         <v>0.69032600659999988</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="5">
         <v>0.64069241300000046</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="5">
         <v>0.80600166799999995</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="5">
         <v>4.8953308599999801E-2</v>
       </c>
-      <c r="J12" s="3">
+      <c r="J12" s="5">
         <v>0.38286439799999972</v>
       </c>
-      <c r="K12" s="3">
+      <c r="K12" s="5">
         <v>0.46240332020000002</v>
       </c>
       <c r="M12">
@@ -4012,31 +4012,31 @@
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="5">
         <v>0.41437519920000021</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="5">
         <v>0.49619987899999968</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="5">
         <v>0.23037171239999979</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="5">
         <v>0.54371098340000046</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="5">
         <v>0.57595649239999958</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="5">
         <v>0.68439392140000033</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="5">
         <v>1.7524141599999599E-2</v>
       </c>
-      <c r="J5" s="3">
+      <c r="J5" s="5">
         <v>0.30865891019999969</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="5">
         <v>0.31845501419999961</v>
       </c>
     </row>
@@ -4044,31 +4044,31 @@
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="5">
         <v>0.62485537820000037</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="5">
         <v>0.62880103120000008</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="5">
         <v>0.38368074000000002</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="5">
         <v>0.65269264039999975</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="5">
         <v>0.66945486279999944</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="5">
         <v>0.68692458160000003</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="5">
         <v>3.2789737000000319E-2</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="5">
         <v>0.43018502259999991</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="5">
         <v>0.1670507846000002</v>
       </c>
     </row>
@@ -4076,31 +4076,31 @@
       <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="5">
         <v>0.40378996460000011</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="5">
         <v>0.2777467598000003</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="5">
         <v>5.6953460200000361E-2</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="5">
         <v>0.41793989259999981</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="5">
         <v>0.34340786800000028</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="5">
         <v>0.45872978119999969</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="5">
         <v>6.1225650000000797E-3</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="5">
         <v>0.18155446079999971</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="5">
         <v>9.5239899999999267E-4</v>
       </c>
     </row>
@@ -4108,31 +4108,31 @@
       <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="5">
         <v>0.55813302540000009</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="5">
         <v>0.34055067100000042</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="5">
         <v>0.11355317219999959</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="5">
         <v>0.52664943560000044</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="5">
         <v>0.42637542660000038</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="5">
         <v>0.58806556539999955</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="5">
         <v>1.687106799999993E-2</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J8" s="5">
         <v>0.25249458060000007</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8" s="5">
         <v>1.2245129999999721E-2</v>
       </c>
     </row>
@@ -4140,31 +4140,31 @@
       <c r="B9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="5">
         <v>5.1320700400000252E-2</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="5">
         <v>0.17486045640000031</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="5">
         <v>4.1905556000001454E-3</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="5">
         <v>0.15238384000000019</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="5">
         <v>0.26800507860000028</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="5">
         <v>0.3292035172000003</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="5">
         <v>1.5510497999997601E-3</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="5">
         <v>5.115743200000189E-3</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="5">
         <v>4.3402182999999983E-2</v>
       </c>
     </row>
@@ -4172,31 +4172,31 @@
       <c r="B10" s="1">
         <v>6</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="5">
         <v>0.1201383309999997</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="5">
         <v>0.14658781179999991</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="5">
         <v>6.0409307999997894E-3</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="5">
         <v>0.19706495880000041</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="5">
         <v>0.21619457300000011</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="5">
         <v>0.28925718200000011</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="5">
         <v>5.2245888000004292E-3</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="5">
         <v>4.7347836000004584E-3</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="5">
         <v>3.8912301999993741E-3</v>
       </c>
     </row>
@@ -4204,31 +4204,31 @@
       <c r="B11" s="1">
         <v>7</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="5">
         <v>6.7266580799999698E-2</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="5">
         <v>6.3647464600000259E-2</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="5">
         <v>1.697991359999973E-2</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="5">
         <v>0.1146144168000003</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="5">
         <v>9.6382778800000235E-2</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="5">
         <v>0.1853368453999997</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="5">
         <v>2.1333737600000461E-2</v>
       </c>
-      <c r="J11" s="3">
+      <c r="J11" s="5">
         <v>1.175532480000019E-2</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="5">
         <v>6.0409308000002326E-3</v>
       </c>
     </row>
@@ -4236,31 +4236,31 @@
       <c r="B12" s="1">
         <v>8</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="5">
         <v>0.67544137079999977</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="5">
         <v>0.63870598080000018</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="5">
         <v>0.37067369080000029</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="5">
         <v>0.71489790080000049</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="5">
         <v>0.69658462860000059</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="5">
         <v>0.81590661760000005</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="5">
         <v>5.5075873599999881E-2</v>
       </c>
-      <c r="J12" s="3">
+      <c r="J12" s="5">
         <v>0.45995429419999972</v>
       </c>
-      <c r="K12" s="3">
+      <c r="K12" s="5">
         <v>0.48077101519999982</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add patameters to the result table
</commit_message>
<xml_diff>
--- a/files/results.xlsx
+++ b/files/results.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" firstSheet="13" activeTab="17"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" firstSheet="15" activeTab="15"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="1" r:id="rId1"/>
@@ -40,13 +40,15 @@
     <sheet name="pbe0 S2_HEOE" sheetId="26" r:id="rId26"/>
     <sheet name="pbe0 T1_HEOE" sheetId="27" r:id="rId27"/>
     <sheet name="pbe0 T2_HEOE" sheetId="28" r:id="rId28"/>
+    <sheet name="pbe0 delta_E_S1_S2" sheetId="29" r:id="rId29"/>
+    <sheet name="pbe0 delta_E_T1_T2" sheetId="30" r:id="rId30"/>
   </sheets>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="45">
   <si>
     <t>Title</t>
   </si>
@@ -175,6 +177,12 @@
   </si>
   <si>
     <t>Hole-electron overlap extent in T2 (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
+    <t>ΔE(S2-S1), eV (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
+    <t>ΔE(T2-T1), eV (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
 </sst>
 </file>
@@ -8794,6 +8802,345 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:K12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="11" width="12.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="20"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="2"/>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.1796331400000039E-2</v>
+      </c>
+      <c r="D5" s="5">
+        <v>4.5334192399999917E-2</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2.612294399999993E-3</v>
+      </c>
+      <c r="F5" s="5">
+        <v>1.251724400000054E-2</v>
+      </c>
+      <c r="G5" s="5">
+        <v>6.2123626199999997E-2</v>
+      </c>
+      <c r="H5" s="5">
+        <v>7.2110209999998176E-3</v>
+      </c>
+      <c r="I5" s="5">
+        <v>2.1224891999995781E-3</v>
+      </c>
+      <c r="J5" s="5">
+        <v>6.4953611800000033E-2</v>
+      </c>
+      <c r="K5" s="5">
+        <v>4.3538239999962869E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="5">
+        <v>1.1918593199999879E-2</v>
+      </c>
+      <c r="D6" s="5">
+        <v>7.2681649400000214E-2</v>
+      </c>
+      <c r="E6" s="5">
+        <v>9.5239899999999267E-4</v>
+      </c>
+      <c r="F6" s="5">
+        <v>2.2313347999998179E-3</v>
+      </c>
+      <c r="G6" s="5">
+        <v>8.0028727399999777E-2</v>
+      </c>
+      <c r="H6" s="5">
+        <v>5.3334343999997813E-3</v>
+      </c>
+      <c r="I6" s="5">
+        <v>2.040855000000175E-3</v>
+      </c>
+      <c r="J6" s="5">
+        <v>0.10623330559999999</v>
+      </c>
+      <c r="K6" s="5">
+        <v>5.1701660000036398E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="5">
+        <v>5.9865079999999793E-2</v>
+      </c>
+      <c r="D7" s="5">
+        <v>6.5851588000000127E-2</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1.469415599999913E-3</v>
+      </c>
+      <c r="F7" s="5">
+        <v>2.7619570999999791E-2</v>
+      </c>
+      <c r="G7" s="5">
+        <v>8.949829460000025E-2</v>
+      </c>
+      <c r="H7" s="5">
+        <v>1.5428863799999529E-2</v>
+      </c>
+      <c r="I7" s="5">
+        <v>1.551049800000204E-3</v>
+      </c>
+      <c r="J7" s="5">
+        <v>8.824657019999993E-2</v>
+      </c>
+      <c r="K7" s="5">
+        <v>2.4490259999998543E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5">
+        <v>0.12753983180000009</v>
+      </c>
+      <c r="D8" s="5">
+        <v>8.1117183400000403E-2</v>
+      </c>
+      <c r="E8" s="5">
+        <v>4.7347836000000143E-3</v>
+      </c>
+      <c r="F8" s="5">
+        <v>8.8137724600000578E-2</v>
+      </c>
+      <c r="G8" s="5">
+        <v>0.1191587206000007</v>
+      </c>
+      <c r="H8" s="5">
+        <v>7.4504813199999465E-2</v>
+      </c>
+      <c r="I8" s="5">
+        <v>7.3470780000000069E-3</v>
+      </c>
+      <c r="J8" s="5">
+        <v>9.932161000000006E-2</v>
+      </c>
+      <c r="K8" s="5">
+        <v>1.074850299999985E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>5</v>
+      </c>
+      <c r="C9" s="5">
+        <v>1.417713940000009E-2</v>
+      </c>
+      <c r="D9" s="5">
+        <v>1.6326840000013829E-4</v>
+      </c>
+      <c r="E9" s="5">
+        <v>3.6463275999998319E-3</v>
+      </c>
+      <c r="F9" s="5">
+        <v>2.3673918000000072E-3</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1.7687410000002399E-3</v>
+      </c>
+      <c r="H9" s="5">
+        <v>1.442204199999964E-3</v>
+      </c>
+      <c r="I9" s="5">
+        <v>1.496626999999862E-3</v>
+      </c>
+      <c r="J9" s="5">
+        <v>4.6531494000001672E-3</v>
+      </c>
+      <c r="K9" s="5">
+        <v>4.6259379999957773E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <v>6</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2.5769195800000141E-2</v>
+      </c>
+      <c r="D10" s="5">
+        <v>7.6191919999990532E-4</v>
+      </c>
+      <c r="E10" s="5">
+        <v>4.1633441999997522E-3</v>
+      </c>
+      <c r="F10" s="5">
+        <v>8.8164936000003635E-3</v>
+      </c>
+      <c r="G10" s="5">
+        <v>4.054498599999512E-3</v>
+      </c>
+      <c r="H10" s="5">
+        <v>3.5374819999978158E-4</v>
+      </c>
+      <c r="I10" s="5">
+        <v>5.1973774000004802E-3</v>
+      </c>
+      <c r="J10" s="5">
+        <v>4.1905556000001454E-3</v>
+      </c>
+      <c r="K10" s="5">
+        <v>3.8640187999994251E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>7</v>
+      </c>
+      <c r="C11" s="5">
+        <v>7.9185173999998248E-3</v>
+      </c>
+      <c r="D11" s="5">
+        <v>8.0817858000004072E-3</v>
+      </c>
+      <c r="E11" s="5">
+        <v>1.5809823399999701E-2</v>
+      </c>
+      <c r="F11" s="5">
+        <v>7.6191919999999413E-3</v>
+      </c>
+      <c r="G11" s="5">
+        <v>3.8640187999998692E-3</v>
+      </c>
+      <c r="H11" s="5">
+        <v>5.7960282000002472E-3</v>
+      </c>
+      <c r="I11" s="5">
+        <v>2.1279314800000119E-2</v>
+      </c>
+      <c r="J11" s="5">
+        <v>1.1455999399999859E-2</v>
+      </c>
+      <c r="K11" s="5">
+        <v>6.0137193999998404E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>8</v>
+      </c>
+      <c r="C12" s="5">
+        <v>6.4327749599999873E-2</v>
+      </c>
+      <c r="D12" s="5">
+        <v>5.096695220000047E-2</v>
+      </c>
+      <c r="E12" s="5">
+        <v>1.9020768599999901E-2</v>
+      </c>
+      <c r="F12" s="5">
+        <v>2.457189420000061E-2</v>
+      </c>
+      <c r="G12" s="5">
+        <v>5.5892215600000128E-2</v>
+      </c>
+      <c r="H12" s="5">
+        <v>9.9049496000001014E-3</v>
+      </c>
+      <c r="I12" s="5">
+        <v>6.1225650000000797E-3</v>
+      </c>
+      <c r="J12" s="5">
+        <v>7.7089896199999952E-2</v>
+      </c>
+      <c r="K12" s="5">
+        <v>1.8367694999999799E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:K2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:K12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:K12"/>
@@ -9125,6 +9472,345 @@
         <cfvo type="max"/>
         <color rgb="FF63BE7B"/>
         <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:K12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="11" width="12.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="20"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="2"/>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>7.2110209999998176E-3</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1.273493520000013E-2</v>
+      </c>
+      <c r="E5" s="5">
+        <v>1.1347153799999621E-2</v>
+      </c>
+      <c r="F5" s="5">
+        <v>7.7552490000005747E-3</v>
+      </c>
+      <c r="G5" s="5">
+        <v>1.6408474199999471E-2</v>
+      </c>
+      <c r="H5" s="5">
+        <v>6.5851588000001024E-3</v>
+      </c>
+      <c r="I5" s="5">
+        <v>2.5306601999997009E-3</v>
+      </c>
+      <c r="J5" s="5">
+        <v>2.949715759999938E-2</v>
+      </c>
+      <c r="K5" s="5">
+        <v>8.1634199999847112E-5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="5">
+        <v>4.3538239999998396E-3</v>
+      </c>
+      <c r="D6" s="5">
+        <v>6.5579474000001534E-3</v>
+      </c>
+      <c r="E6" s="5">
+        <v>6.0137193999998404E-3</v>
+      </c>
+      <c r="F6" s="5">
+        <v>3.619116200000327E-3</v>
+      </c>
+      <c r="G6" s="5">
+        <v>1.0068217999999801E-2</v>
+      </c>
+      <c r="H6" s="5">
+        <v>3.972864400000109E-3</v>
+      </c>
+      <c r="I6" s="5">
+        <v>2.6939286000002842E-3</v>
+      </c>
+      <c r="J6" s="5">
+        <v>3.0204653999999831E-2</v>
+      </c>
+      <c r="K6" s="5">
+        <v>5.4422799999898068E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="5">
+        <v>5.1973774000000361E-3</v>
+      </c>
+      <c r="D7" s="5">
+        <v>8.8981278000002106E-3</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1.22995528000005E-2</v>
+      </c>
+      <c r="F7" s="5">
+        <v>3.7823846000000221E-3</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1.1864170400000431E-2</v>
+      </c>
+      <c r="H7" s="5">
+        <v>3.5102706000000872E-3</v>
+      </c>
+      <c r="I7" s="5">
+        <v>1.6054726000001021E-3</v>
+      </c>
+      <c r="J7" s="5">
+        <v>5.4939816599999691E-2</v>
+      </c>
+      <c r="K7" s="5">
+        <v>2.1769120000003639E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5">
+        <v>1.099340560000028E-2</v>
+      </c>
+      <c r="D8" s="5">
+        <v>1.24083984000003E-2</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2.6231789599999718E-2</v>
+      </c>
+      <c r="F8" s="5">
+        <v>7.3198666000000578E-3</v>
+      </c>
+      <c r="G8" s="5">
+        <v>2.3864397800000159E-2</v>
+      </c>
+      <c r="H8" s="5">
+        <v>1.7959523999997451E-3</v>
+      </c>
+      <c r="I8" s="5">
+        <v>7.8368831999999777E-3</v>
+      </c>
+      <c r="J8" s="5">
+        <v>6.6994466799999763E-2</v>
+      </c>
+      <c r="K8" s="5">
+        <v>1.07212915999999E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>5</v>
+      </c>
+      <c r="C9" s="5">
+        <v>1.2925415000000219E-2</v>
+      </c>
+      <c r="D9" s="5">
+        <v>1.213628440000036E-2</v>
+      </c>
+      <c r="E9" s="5">
+        <v>3.4830592000001381E-3</v>
+      </c>
+      <c r="F9" s="5">
+        <v>2.7483514000001819E-3</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1.4476464799999981E-2</v>
+      </c>
+      <c r="H9" s="5">
+        <v>4.8708406000002036E-3</v>
+      </c>
+      <c r="I9" s="5">
+        <v>1.496626999999862E-3</v>
+      </c>
+      <c r="J9" s="5">
+        <v>4.544303799999927E-3</v>
+      </c>
+      <c r="K9" s="5">
+        <v>1.360570000001893E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <v>6</v>
+      </c>
+      <c r="C10" s="5">
+        <v>1.896634580000001E-2</v>
+      </c>
+      <c r="D10" s="5">
+        <v>5.8776623999996502E-3</v>
+      </c>
+      <c r="E10" s="5">
+        <v>3.6463275999998319E-3</v>
+      </c>
+      <c r="F10" s="5">
+        <v>9.5512014000003198E-3</v>
+      </c>
+      <c r="G10" s="5">
+        <v>4.3810354000002327E-3</v>
+      </c>
+      <c r="H10" s="5">
+        <v>4.0544985999999561E-3</v>
+      </c>
+      <c r="I10" s="5">
+        <v>5.1973774000004802E-3</v>
+      </c>
+      <c r="J10" s="5">
+        <v>4.0817100000003492E-3</v>
+      </c>
+      <c r="K10" s="5">
+        <v>3.8640187999994251E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>7</v>
+      </c>
+      <c r="C11" s="5">
+        <v>5.3334343999997813E-3</v>
+      </c>
+      <c r="D11" s="5">
+        <v>9.687258400000065E-3</v>
+      </c>
+      <c r="E11" s="5">
+        <v>1.5456075199999921E-2</v>
+      </c>
+      <c r="F11" s="5">
+        <v>8.1362086000003053E-3</v>
+      </c>
+      <c r="G11" s="5">
+        <v>4.7347836000004584E-3</v>
+      </c>
+      <c r="H11" s="5">
+        <v>1.104782839999929E-2</v>
+      </c>
+      <c r="I11" s="5">
+        <v>2.1306526200000508E-2</v>
+      </c>
+      <c r="J11" s="5">
+        <v>1.142878800000036E-2</v>
+      </c>
+      <c r="K11" s="5">
+        <v>6.0409308000002326E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>8</v>
+      </c>
+      <c r="C12" s="5">
+        <v>4.4354582000001308E-3</v>
+      </c>
+      <c r="D12" s="5">
+        <v>6.5307359999997594E-3</v>
+      </c>
+      <c r="E12" s="5">
+        <v>1.058523460000016E-2</v>
+      </c>
+      <c r="F12" s="5">
+        <v>3.755173200000073E-3</v>
+      </c>
+      <c r="G12" s="5">
+        <v>8.489956800000531E-3</v>
+      </c>
+      <c r="H12" s="5">
+        <v>8.7076480000001233E-3</v>
+      </c>
+      <c r="I12" s="5">
+        <v>5.7416054000003491E-3</v>
+      </c>
+      <c r="J12" s="5">
+        <v>1.553770940000021E-2</v>
+      </c>
+      <c r="K12" s="5">
+        <v>2.7211399999993452E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:K2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:K12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
add S2 and T2 energies to results.xls
</commit_message>
<xml_diff>
--- a/files/results.xlsx
+++ b/files/results.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" firstSheet="15" activeTab="18"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" firstSheet="17" activeTab="31"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="1" r:id="rId1"/>
@@ -42,13 +42,15 @@
     <sheet name="pbe0 T2_HEOE" sheetId="28" r:id="rId28"/>
     <sheet name="pbe0 delta_E_S1_S2" sheetId="29" r:id="rId29"/>
     <sheet name="pbe0 delta_E_T1_T2" sheetId="30" r:id="rId30"/>
+    <sheet name="pbe0 S2_energy" sheetId="31" r:id="rId31"/>
+    <sheet name="pbe0 T2_energy" sheetId="32" r:id="rId32"/>
   </sheets>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="51">
   <si>
     <t>Title</t>
   </si>
@@ -131,10 +133,10 @@
     <t>ΔE(S2-T1), eV (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
-    <t>Spin-Orbit Coupling Matrix Element for S1 and T1, cm-1 (PBE0/def2-TZVP, CPCM(toluene))</t>
+    <t>Spin-Orbit Coupling Matrix Element between S1 and T1, cm-1 (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
-    <t>Spin-Orbit Coupling between T1 and S2, cm-1 (PBE0/def2-TZVP, CPCM(toluene))</t>
+    <t>Spin-Orbit Coupling Matrix Element between T1 and S2, cm-1 (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
     <t>(SOCME(T1-S1))^2*exp(-ΔE(S1-T1)^2) (PBE0/def2-TZVP, CPCM(toluene))</t>
@@ -161,7 +163,7 @@
     <t>Distance between centroids of HOMO and LUMO (PBE0/def2-TZVP, CPCM(toluene)), Angstrom</t>
   </si>
   <si>
-    <t>Overlap integral for module of HOMO and LUMO (PBE0/def2-TZVP, CPCM(toluene))</t>
+    <t>Overlap integral of HOMO and LUMO modules (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
     <t>Overlap integral for squared HOMO and LUMO (PBE0/def2-TZVP, CPCM(toluene))</t>
@@ -170,19 +172,37 @@
     <t>Hole-electron overlap extent in S1 (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
+    <t>Contribution of LE character for S1, % (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
     <t>Hole-electron overlap extent in S2 (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
+    <t>Contribution of LE character for S2, % (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
     <t>Hole-electron overlap extent in T1 (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
+    <t>Contribution of LE character for T1, % (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
     <t>Hole-electron overlap extent in T2 (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
+    <t>Contribution of LE character for T2, % (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
     <t>ΔE(S2-S1), eV (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
   <si>
     <t>ΔE(T2-T1), eV (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
+    <t>S2 energies, eV (PBE0/def2-TZVP, CPCM(toluene))</t>
+  </si>
+  <si>
+    <t>T2 energies, eV (PBE0/def2-TZVP, CPCM(toluene))</t>
   </si>
 </sst>
 </file>
@@ -226,7 +246,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -279,6 +299,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD7D7D7"/>
         <bgColor rgb="FFD7D7D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -413,7 +445,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -444,6 +476,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -467,6 +502,16 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -778,18 +823,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -973,18 +1018,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -1312,18 +1357,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -1720,18 +1765,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -2107,18 +2152,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -2508,18 +2553,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -2847,18 +2892,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -3197,18 +3242,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:23" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -3961,18 +4006,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -4300,18 +4345,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -4649,18 +4694,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -4988,18 +5033,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -5327,18 +5372,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -5842,18 +5887,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -6357,18 +6402,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -6696,18 +6741,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -7126,18 +7171,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -7448,25 +7493,25 @@
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:K26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -7766,17 +7811,412 @@
         <v>2.525816935377876E-3</v>
       </c>
     </row>
+    <row r="16" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="21"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+    </row>
+    <row r="18" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" s="18">
+        <f t="shared" ref="C19:K19" si="0">C5*100</f>
+        <v>12.29031228527476</v>
+      </c>
+      <c r="D19" s="18">
+        <f t="shared" si="0"/>
+        <v>7.7732857119534371</v>
+      </c>
+      <c r="E19" s="18">
+        <f t="shared" si="0"/>
+        <v>0.90012866724608442</v>
+      </c>
+      <c r="F19" s="18">
+        <f t="shared" si="0"/>
+        <v>14.292783138867049</v>
+      </c>
+      <c r="G19" s="18">
+        <f t="shared" si="0"/>
+        <v>10.38004605117753</v>
+      </c>
+      <c r="H19" s="18">
+        <f t="shared" si="0"/>
+        <v>16.929496135528861</v>
+      </c>
+      <c r="I19" s="18">
+        <f t="shared" si="0"/>
+        <v>0.36982715595790711</v>
+      </c>
+      <c r="J19" s="18">
+        <f t="shared" si="0"/>
+        <v>4.1400177995625214</v>
+      </c>
+      <c r="K19" s="18">
+        <f t="shared" si="0"/>
+        <v>8.6403054635793397E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="18">
+        <f t="shared" ref="C20:K20" si="1">C6*100</f>
+        <v>41.011389342832274</v>
+      </c>
+      <c r="D20" s="18">
+        <f t="shared" si="1"/>
+        <v>15.1574142632183</v>
+      </c>
+      <c r="E20" s="18">
+        <f t="shared" si="1"/>
+        <v>2.096115033592381</v>
+      </c>
+      <c r="F20" s="18">
+        <f t="shared" si="1"/>
+        <v>42.816434057439118</v>
+      </c>
+      <c r="G20" s="18">
+        <f t="shared" si="1"/>
+        <v>17.716605250935221</v>
+      </c>
+      <c r="H20" s="18">
+        <f t="shared" si="1"/>
+        <v>44.271140909825853</v>
+      </c>
+      <c r="I20" s="18">
+        <f t="shared" si="1"/>
+        <v>0.7045688536189415</v>
+      </c>
+      <c r="J20" s="18">
+        <f t="shared" si="1"/>
+        <v>13.101842079110741</v>
+      </c>
+      <c r="K20" s="18">
+        <f t="shared" si="1"/>
+        <v>0.25583055678211281</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1">
+        <v>3</v>
+      </c>
+      <c r="C21" s="18">
+        <f t="shared" ref="C21:K21" si="2">C7*100</f>
+        <v>15.7348262078342</v>
+      </c>
+      <c r="D21" s="18">
+        <f t="shared" si="2"/>
+        <v>5.0985279592860229</v>
+      </c>
+      <c r="E21" s="18">
+        <f t="shared" si="2"/>
+        <v>1.0666595742502121</v>
+      </c>
+      <c r="F21" s="18">
+        <f t="shared" si="2"/>
+        <v>10.434114034040611</v>
+      </c>
+      <c r="G21" s="18">
+        <f t="shared" si="2"/>
+        <v>6.0757850543438821</v>
+      </c>
+      <c r="H21" s="18">
+        <f t="shared" si="2"/>
+        <v>25.222998159089236</v>
+      </c>
+      <c r="I21" s="18">
+        <f t="shared" si="2"/>
+        <v>0.17654848775081791</v>
+      </c>
+      <c r="J21" s="18">
+        <f t="shared" si="2"/>
+        <v>4.8290913860019238</v>
+      </c>
+      <c r="K21" s="18">
+        <f t="shared" si="2"/>
+        <v>8.2749241156752418E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>4</v>
+      </c>
+      <c r="C22" s="18">
+        <f t="shared" ref="C22:K22" si="3">C8*100</f>
+        <v>11.433896432845431</v>
+      </c>
+      <c r="D22" s="18">
+        <f t="shared" si="3"/>
+        <v>9.1055458946078272</v>
+      </c>
+      <c r="E22" s="18">
+        <f t="shared" si="3"/>
+        <v>1.3015868282772149</v>
+      </c>
+      <c r="F22" s="18">
+        <f t="shared" si="3"/>
+        <v>9.9127906478584791</v>
+      </c>
+      <c r="G22" s="18">
+        <f t="shared" si="3"/>
+        <v>10.5471923134376</v>
+      </c>
+      <c r="H22" s="18">
+        <f t="shared" si="3"/>
+        <v>13.08058231168804</v>
+      </c>
+      <c r="I22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.32272822023779602</v>
+      </c>
+      <c r="J22" s="18">
+        <f t="shared" si="3"/>
+        <v>7.6693147641236772</v>
+      </c>
+      <c r="K22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.1421146158968839</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="1">
+        <v>5</v>
+      </c>
+      <c r="C23" s="18">
+        <f t="shared" ref="C23:K23" si="4">C9*100</f>
+        <v>4.2113131794149385</v>
+      </c>
+      <c r="D23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.93140719458949506</v>
+      </c>
+      <c r="E23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.1247946573099689</v>
+      </c>
+      <c r="F23" s="18">
+        <f t="shared" si="4"/>
+        <v>4.8424730880020528</v>
+      </c>
+      <c r="G23" s="18">
+        <f t="shared" si="4"/>
+        <v>1.1205192975266129</v>
+      </c>
+      <c r="H23" s="18">
+        <f t="shared" si="4"/>
+        <v>5.2161581264746699</v>
+      </c>
+      <c r="I23" s="18">
+        <f t="shared" si="4"/>
+        <v>2.393274682723796E-2</v>
+      </c>
+      <c r="J23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.3315058616646237</v>
+      </c>
+      <c r="K23" s="18">
+        <f t="shared" si="4"/>
+        <v>1.3477327378624971E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="1">
+        <v>6</v>
+      </c>
+      <c r="C24" s="18">
+        <f t="shared" ref="C24:K24" si="5">C10*100</f>
+        <v>4.2518264585621042</v>
+      </c>
+      <c r="D24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.709583923058813</v>
+      </c>
+      <c r="E24" s="18">
+        <f t="shared" si="5"/>
+        <v>0.11332614224961091</v>
+      </c>
+      <c r="F24" s="18">
+        <f t="shared" si="5"/>
+        <v>9.6903802067274469</v>
+      </c>
+      <c r="G24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.964513849788883</v>
+      </c>
+      <c r="H24" s="18">
+        <f t="shared" si="5"/>
+        <v>13.577237886891819</v>
+      </c>
+      <c r="I24" s="18">
+        <f t="shared" si="5"/>
+        <v>2.2463611284649538E-2</v>
+      </c>
+      <c r="J24" s="18">
+        <f t="shared" si="5"/>
+        <v>0.2347892918685153</v>
+      </c>
+      <c r="K24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.2577966054055841E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="1">
+        <v>7</v>
+      </c>
+      <c r="C25" s="18">
+        <f t="shared" ref="C25:K25" si="6">C11*100</f>
+        <v>4.1735247513627973</v>
+      </c>
+      <c r="D25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.0886834159234291</v>
+      </c>
+      <c r="E25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.11975539175296711</v>
+      </c>
+      <c r="F25" s="18">
+        <f t="shared" si="6"/>
+        <v>4.9987079394581428</v>
+      </c>
+      <c r="G25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.212486066291943</v>
+      </c>
+      <c r="H25" s="18">
+        <f t="shared" si="6"/>
+        <v>5.7627513361363754</v>
+      </c>
+      <c r="I25" s="18">
+        <f t="shared" si="6"/>
+        <v>2.400669017848998E-2</v>
+      </c>
+      <c r="J25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.28681161559362589</v>
+      </c>
+      <c r="K25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.3307778620332071E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="1">
+        <v>8</v>
+      </c>
+      <c r="C26" s="18">
+        <f t="shared" ref="C26:K26" si="7">C12*100</f>
+        <v>19.891121812027958</v>
+      </c>
+      <c r="D26" s="18">
+        <f t="shared" si="7"/>
+        <v>16.848204255293101</v>
+      </c>
+      <c r="E26" s="18">
+        <f t="shared" si="7"/>
+        <v>1.6504890030350321</v>
+      </c>
+      <c r="F26" s="18">
+        <f t="shared" si="7"/>
+        <v>23.54288680857406</v>
+      </c>
+      <c r="G26" s="18">
+        <f t="shared" si="7"/>
+        <v>20.024322945037522</v>
+      </c>
+      <c r="H26" s="18">
+        <f t="shared" si="7"/>
+        <v>36.537661507793118</v>
+      </c>
+      <c r="I26" s="18">
+        <f t="shared" si="7"/>
+        <v>1.1322842649085241</v>
+      </c>
+      <c r="J26" s="18">
+        <f t="shared" si="7"/>
+        <v>14.14258524591879</v>
+      </c>
+      <c r="K26" s="18">
+        <f t="shared" si="7"/>
+        <v>0.25258169353778759</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B16:K16"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:K12">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19:K26">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color theme="0"/>
+        <color theme="3" tint="0.39997558519241921"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -7787,25 +8227,25 @@
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:K26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="B2" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -8105,17 +8545,412 @@
         <v>2.682923382755466E-3</v>
       </c>
     </row>
+    <row r="16" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="21"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+    </row>
+    <row r="18" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" s="18">
+        <f t="shared" ref="C19:K19" si="0">C5*100</f>
+        <v>12.400345455585569</v>
+      </c>
+      <c r="D19" s="18">
+        <f t="shared" si="0"/>
+        <v>7.9891583356523759</v>
+      </c>
+      <c r="E19" s="18">
+        <f t="shared" si="0"/>
+        <v>0.81031199347937866</v>
+      </c>
+      <c r="F19" s="18">
+        <f t="shared" si="0"/>
+        <v>14.04182515218614</v>
+      </c>
+      <c r="G19" s="18">
+        <f t="shared" si="0"/>
+        <v>11.67876314882448</v>
+      </c>
+      <c r="H19" s="18">
+        <f t="shared" si="0"/>
+        <v>16.52412204057741</v>
+      </c>
+      <c r="I19" s="18">
+        <f t="shared" si="0"/>
+        <v>0.36175782767151449</v>
+      </c>
+      <c r="J19" s="18">
+        <f t="shared" si="0"/>
+        <v>4.3550542641768182</v>
+      </c>
+      <c r="K19" s="18">
+        <f t="shared" si="0"/>
+        <v>8.6950302615110026E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="18">
+        <f t="shared" ref="C20:K20" si="1">C6*100</f>
+        <v>41.6539752607083</v>
+      </c>
+      <c r="D20" s="18">
+        <f t="shared" si="1"/>
+        <v>21.114469236109208</v>
+      </c>
+      <c r="E20" s="18">
+        <f t="shared" si="1"/>
+        <v>2.0403575219639341</v>
+      </c>
+      <c r="F20" s="18">
+        <f t="shared" si="1"/>
+        <v>42.374555594815568</v>
+      </c>
+      <c r="G20" s="18">
+        <f t="shared" si="1"/>
+        <v>37.19867055091752</v>
+      </c>
+      <c r="H20" s="18">
+        <f t="shared" si="1"/>
+        <v>44.679363022133487</v>
+      </c>
+      <c r="I20" s="18">
+        <f t="shared" si="1"/>
+        <v>0.69697110935283257</v>
+      </c>
+      <c r="J20" s="18">
+        <f t="shared" si="1"/>
+        <v>13.037966666350789</v>
+      </c>
+      <c r="K20" s="18">
+        <f t="shared" si="1"/>
+        <v>0.25674769153019089</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1">
+        <v>3</v>
+      </c>
+      <c r="C21" s="18">
+        <f t="shared" ref="C21:K21" si="2">C7*100</f>
+        <v>24.566852440787802</v>
+      </c>
+      <c r="D21" s="18">
+        <f t="shared" si="2"/>
+        <v>6.4640996761773799</v>
+      </c>
+      <c r="E21" s="18">
+        <f t="shared" si="2"/>
+        <v>0.9689240369749752</v>
+      </c>
+      <c r="F21" s="18">
+        <f t="shared" si="2"/>
+        <v>25.561023559097791</v>
+      </c>
+      <c r="G21" s="18">
+        <f t="shared" si="2"/>
+        <v>9.1385041776418632</v>
+      </c>
+      <c r="H21" s="18">
+        <f t="shared" si="2"/>
+        <v>26.726840122494139</v>
+      </c>
+      <c r="I21" s="18">
+        <f t="shared" si="2"/>
+        <v>0.17521874845047761</v>
+      </c>
+      <c r="J21" s="18">
+        <f t="shared" si="2"/>
+        <v>5.7395710384093288</v>
+      </c>
+      <c r="K21" s="18">
+        <f t="shared" si="2"/>
+        <v>8.2627958451535213E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>4</v>
+      </c>
+      <c r="C22" s="18">
+        <f t="shared" ref="C22:K22" si="3">C8*100</f>
+        <v>30.551666115764942</v>
+      </c>
+      <c r="D22" s="18">
+        <f t="shared" si="3"/>
+        <v>9.646822105840906</v>
+      </c>
+      <c r="E22" s="18">
+        <f t="shared" si="3"/>
+        <v>1.3772117351787501</v>
+      </c>
+      <c r="F22" s="18">
+        <f t="shared" si="3"/>
+        <v>12.44038093615185</v>
+      </c>
+      <c r="G22" s="18">
+        <f t="shared" si="3"/>
+        <v>12.796704640288409</v>
+      </c>
+      <c r="H22" s="18">
+        <f t="shared" si="3"/>
+        <v>26.256824784474247</v>
+      </c>
+      <c r="I22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.30979810655302148</v>
+      </c>
+      <c r="J22" s="18">
+        <f t="shared" si="3"/>
+        <v>8.244023287681765</v>
+      </c>
+      <c r="K22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.1375471084140249</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="1">
+        <v>5</v>
+      </c>
+      <c r="C23" s="18">
+        <f t="shared" ref="C23:K23" si="4">C9*100</f>
+        <v>4.2364926084781027</v>
+      </c>
+      <c r="D23" s="18">
+        <f t="shared" si="4"/>
+        <v>1.2939349945923619</v>
+      </c>
+      <c r="E23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.14559807140528389</v>
+      </c>
+      <c r="F23" s="18">
+        <f t="shared" si="4"/>
+        <v>4.8163629461499911</v>
+      </c>
+      <c r="G23" s="18">
+        <f t="shared" si="4"/>
+        <v>1.122245732281216</v>
+      </c>
+      <c r="H23" s="18">
+        <f t="shared" si="4"/>
+        <v>5.1632051538621955</v>
+      </c>
+      <c r="I23" s="18">
+        <f t="shared" si="4"/>
+        <v>2.4005926346486069E-2</v>
+      </c>
+      <c r="J23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.28443568223188054</v>
+      </c>
+      <c r="K23" s="18">
+        <f t="shared" si="4"/>
+        <v>1.356850530552008E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="1">
+        <v>6</v>
+      </c>
+      <c r="C24" s="18">
+        <f t="shared" ref="C24:K24" si="5">C10*100</f>
+        <v>4.0696205989793173</v>
+      </c>
+      <c r="D24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.6439613710401102</v>
+      </c>
+      <c r="E24" s="18">
+        <f t="shared" si="5"/>
+        <v>0.13197810035930699</v>
+      </c>
+      <c r="F24" s="18">
+        <f t="shared" si="5"/>
+        <v>9.5178543767649959</v>
+      </c>
+      <c r="G24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.9189874797968891</v>
+      </c>
+      <c r="H24" s="18">
+        <f t="shared" si="5"/>
+        <v>14.193066458270319</v>
+      </c>
+      <c r="I24" s="18">
+        <f t="shared" si="5"/>
+        <v>2.2651045995370499E-2</v>
+      </c>
+      <c r="J24" s="18">
+        <f t="shared" si="5"/>
+        <v>0.2906156144169551</v>
+      </c>
+      <c r="K24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.264620534031086E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="1">
+        <v>7</v>
+      </c>
+      <c r="C25" s="18">
+        <f t="shared" ref="C25:K25" si="6">C11*100</f>
+        <v>4.2187447230884958</v>
+      </c>
+      <c r="D25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.3904211744045369</v>
+      </c>
+      <c r="E25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.13687176247641669</v>
+      </c>
+      <c r="F25" s="18">
+        <f t="shared" si="6"/>
+        <v>5.0134612356309463</v>
+      </c>
+      <c r="G25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.115149594009224</v>
+      </c>
+      <c r="H25" s="18">
+        <f t="shared" si="6"/>
+        <v>5.6879483657361369</v>
+      </c>
+      <c r="I25" s="18">
+        <f t="shared" si="6"/>
+        <v>2.37658334706254E-2</v>
+      </c>
+      <c r="J25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.28296694993559296</v>
+      </c>
+      <c r="K25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.3319339110013319E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="1">
+        <v>8</v>
+      </c>
+      <c r="C26" s="18">
+        <f t="shared" ref="C26:K26" si="7">C12*100</f>
+        <v>32.962431511301524</v>
+      </c>
+      <c r="D26" s="18">
+        <f t="shared" si="7"/>
+        <v>22.21545914874368</v>
+      </c>
+      <c r="E26" s="18">
+        <f t="shared" si="7"/>
+        <v>2.0079508815007849</v>
+      </c>
+      <c r="F26" s="18">
+        <f t="shared" si="7"/>
+        <v>24.7088508675645</v>
+      </c>
+      <c r="G26" s="18">
+        <f t="shared" si="7"/>
+        <v>27.771428907974698</v>
+      </c>
+      <c r="H26" s="18">
+        <f t="shared" si="7"/>
+        <v>35.290074448822573</v>
+      </c>
+      <c r="I26" s="18">
+        <f t="shared" si="7"/>
+        <v>1.1192415189498361</v>
+      </c>
+      <c r="J26" s="18">
+        <f t="shared" si="7"/>
+        <v>17.308509887195331</v>
+      </c>
+      <c r="K26" s="18">
+        <f t="shared" si="7"/>
+        <v>0.2682923382755466</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B16:K16"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:K12">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19:K26">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color theme="0"/>
+        <color theme="3" tint="0.39997558519241921"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -8126,25 +8961,25 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:K26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="B2" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -8444,17 +9279,412 @@
         <v>0.61105844753107841</v>
       </c>
     </row>
+    <row r="16" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="21"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+    </row>
+    <row r="18" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" s="18">
+        <f t="shared" ref="C19:K19" si="0">C5*100</f>
+        <v>52.28354340864653</v>
+      </c>
+      <c r="D19" s="18">
+        <f t="shared" si="0"/>
+        <v>59.685141627224233</v>
+      </c>
+      <c r="E19" s="18">
+        <f t="shared" si="0"/>
+        <v>58.345365045853526</v>
+      </c>
+      <c r="F19" s="18">
+        <f t="shared" si="0"/>
+        <v>59.952575026711855</v>
+      </c>
+      <c r="G19" s="18">
+        <f t="shared" si="0"/>
+        <v>61.098867500910423</v>
+      </c>
+      <c r="H19" s="18">
+        <f t="shared" si="0"/>
+        <v>63.585869154911848</v>
+      </c>
+      <c r="I19" s="18">
+        <f t="shared" si="0"/>
+        <v>0.72482670419594875</v>
+      </c>
+      <c r="J19" s="18">
+        <f t="shared" si="0"/>
+        <v>46.745390981540581</v>
+      </c>
+      <c r="K19" s="18">
+        <f t="shared" si="0"/>
+        <v>60.985989132962374</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="18">
+        <f t="shared" ref="C20:K20" si="1">C6*100</f>
+        <v>51.760198891227546</v>
+      </c>
+      <c r="D20" s="18">
+        <f t="shared" si="1"/>
+        <v>56.30323973332262</v>
+      </c>
+      <c r="E20" s="18">
+        <f t="shared" si="1"/>
+        <v>52.56200305085256</v>
+      </c>
+      <c r="F20" s="18">
+        <f t="shared" si="1"/>
+        <v>52.699162178146729</v>
+      </c>
+      <c r="G20" s="18">
+        <f t="shared" si="1"/>
+        <v>56.657541792742585</v>
+      </c>
+      <c r="H20" s="18">
+        <f t="shared" si="1"/>
+        <v>56.08234670515229</v>
+      </c>
+      <c r="I20" s="18">
+        <f t="shared" si="1"/>
+        <v>2.3244140539810121</v>
+      </c>
+      <c r="J20" s="18">
+        <f t="shared" si="1"/>
+        <v>46.593132262096731</v>
+      </c>
+      <c r="K20" s="18">
+        <f t="shared" si="1"/>
+        <v>61.823174812132351</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1">
+        <v>3</v>
+      </c>
+      <c r="C21" s="18">
+        <f t="shared" ref="C21:K21" si="2">C7*100</f>
+        <v>38.85566900235591</v>
+      </c>
+      <c r="D21" s="18">
+        <f t="shared" si="2"/>
+        <v>44.110136755014416</v>
+      </c>
+      <c r="E21" s="18">
+        <f t="shared" si="2"/>
+        <v>30.287036675369126</v>
+      </c>
+      <c r="F21" s="18">
+        <f t="shared" si="2"/>
+        <v>41.59277510228209</v>
+      </c>
+      <c r="G21" s="18">
+        <f t="shared" si="2"/>
+        <v>48.968314053238018</v>
+      </c>
+      <c r="H21" s="18">
+        <f t="shared" si="2"/>
+        <v>50.845347995277265</v>
+      </c>
+      <c r="I21" s="18">
+        <f t="shared" si="2"/>
+        <v>0.17690258468198822</v>
+      </c>
+      <c r="J21" s="18">
+        <f t="shared" si="2"/>
+        <v>15.6430064485976</v>
+      </c>
+      <c r="K21" s="18">
+        <f t="shared" si="2"/>
+        <v>8.2733763772874197E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>4</v>
+      </c>
+      <c r="C22" s="18">
+        <f t="shared" ref="C22:K22" si="3">C8*100</f>
+        <v>40.311414390392891</v>
+      </c>
+      <c r="D22" s="18">
+        <f t="shared" si="3"/>
+        <v>46.542126561476721</v>
+      </c>
+      <c r="E22" s="18">
+        <f t="shared" si="3"/>
+        <v>38.119601527267449</v>
+      </c>
+      <c r="F22" s="18">
+        <f t="shared" si="3"/>
+        <v>46.986984958463879</v>
+      </c>
+      <c r="G22" s="18">
+        <f t="shared" si="3"/>
+        <v>43.592362327181824</v>
+      </c>
+      <c r="H22" s="18">
+        <f t="shared" si="3"/>
+        <v>46.828188894333799</v>
+      </c>
+      <c r="I22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.32286233486277111</v>
+      </c>
+      <c r="J22" s="18">
+        <f t="shared" si="3"/>
+        <v>20.714819843295292</v>
+      </c>
+      <c r="K22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.14211461772514908</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="1">
+        <v>5</v>
+      </c>
+      <c r="C23" s="18">
+        <f t="shared" ref="C23:K23" si="4">C9*100</f>
+        <v>6.8815829507451127</v>
+      </c>
+      <c r="D23" s="18">
+        <f t="shared" si="4"/>
+        <v>60.419834052883623</v>
+      </c>
+      <c r="E23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.1248187051340917</v>
+      </c>
+      <c r="F23" s="18">
+        <f t="shared" si="4"/>
+        <v>62.370031841847904</v>
+      </c>
+      <c r="G23" s="18">
+        <f t="shared" si="4"/>
+        <v>60.599553552438223</v>
+      </c>
+      <c r="H23" s="18">
+        <f t="shared" si="4"/>
+        <v>66.721088473129683</v>
+      </c>
+      <c r="I23" s="18">
+        <f t="shared" si="4"/>
+        <v>2.393276278706832E-2</v>
+      </c>
+      <c r="J23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.3324442342571961</v>
+      </c>
+      <c r="K23" s="18">
+        <f t="shared" si="4"/>
+        <v>60.927114237010116</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="1">
+        <v>6</v>
+      </c>
+      <c r="C24" s="18">
+        <f t="shared" ref="C24:K24" si="5">C10*100</f>
+        <v>27.41459709340031</v>
+      </c>
+      <c r="D24" s="18">
+        <f t="shared" si="5"/>
+        <v>37.428645423458548</v>
+      </c>
+      <c r="E24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.9265231711508339</v>
+      </c>
+      <c r="F24" s="18">
+        <f t="shared" si="5"/>
+        <v>36.910477189708338</v>
+      </c>
+      <c r="G24" s="18">
+        <f t="shared" si="5"/>
+        <v>39.244141334176682</v>
+      </c>
+      <c r="H24" s="18">
+        <f t="shared" si="5"/>
+        <v>40.126553480490692</v>
+      </c>
+      <c r="I24" s="18">
+        <f t="shared" si="5"/>
+        <v>2.2463611786009318E-2</v>
+      </c>
+      <c r="J24" s="18">
+        <f t="shared" si="5"/>
+        <v>0.2411226004708325</v>
+      </c>
+      <c r="K24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.2577966228032839E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="1">
+        <v>7</v>
+      </c>
+      <c r="C25" s="18">
+        <f t="shared" ref="C25:K25" si="6">C11*100</f>
+        <v>14.46562995293568</v>
+      </c>
+      <c r="D25" s="18">
+        <f t="shared" si="6"/>
+        <v>30.143078781629228</v>
+      </c>
+      <c r="E25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.1197914110456058</v>
+      </c>
+      <c r="F25" s="18">
+        <f t="shared" si="6"/>
+        <v>28.656285449762642</v>
+      </c>
+      <c r="G25" s="18">
+        <f t="shared" si="6"/>
+        <v>38.911392866667569</v>
+      </c>
+      <c r="H25" s="18">
+        <f t="shared" si="6"/>
+        <v>40.902728828858947</v>
+      </c>
+      <c r="I25" s="18">
+        <f t="shared" si="6"/>
+        <v>2.400668841424267E-2</v>
+      </c>
+      <c r="J25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.28811872629870627</v>
+      </c>
+      <c r="K25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.3307778655092341E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="1">
+        <v>8</v>
+      </c>
+      <c r="C26" s="18">
+        <f t="shared" ref="C26:K26" si="7">C12*100</f>
+        <v>51.160464790969741</v>
+      </c>
+      <c r="D26" s="18">
+        <f t="shared" si="7"/>
+        <v>62.32679274861308</v>
+      </c>
+      <c r="E26" s="18">
+        <f t="shared" si="7"/>
+        <v>54.815999335857889</v>
+      </c>
+      <c r="F26" s="18">
+        <f t="shared" si="7"/>
+        <v>58.54061283642524</v>
+      </c>
+      <c r="G26" s="18">
+        <f t="shared" si="7"/>
+        <v>61.764022824871255</v>
+      </c>
+      <c r="H26" s="18">
+        <f t="shared" si="7"/>
+        <v>62.151680980273646</v>
+      </c>
+      <c r="I26" s="18">
+        <f t="shared" si="7"/>
+        <v>4.5493819341109427</v>
+      </c>
+      <c r="J26" s="18">
+        <f t="shared" si="7"/>
+        <v>51.269689331705727</v>
+      </c>
+      <c r="K26" s="18">
+        <f t="shared" si="7"/>
+        <v>61.105844753107839</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B16:K16"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:K12">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19:K26">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color theme="0"/>
+        <color theme="3" tint="0.39997558519241921"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -8465,25 +9695,25 @@
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:K26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="B2" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -8783,17 +10013,412 @@
         <v>0.61260249678497058</v>
       </c>
     </row>
+    <row r="16" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="21"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+    </row>
+    <row r="18" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" s="18">
+        <f t="shared" ref="C19:K19" si="0">C5*100</f>
+        <v>55.372940557994497</v>
+      </c>
+      <c r="D19" s="18">
+        <f t="shared" si="0"/>
+        <v>62.945326267629177</v>
+      </c>
+      <c r="E19" s="18">
+        <f t="shared" si="0"/>
+        <v>60.382317166873548</v>
+      </c>
+      <c r="F19" s="18">
+        <f t="shared" si="0"/>
+        <v>60.344611451198645</v>
+      </c>
+      <c r="G19" s="18">
+        <f t="shared" si="0"/>
+        <v>63.028903611695867</v>
+      </c>
+      <c r="H19" s="18">
+        <f t="shared" si="0"/>
+        <v>64.699909438751973</v>
+      </c>
+      <c r="I19" s="18">
+        <f t="shared" si="0"/>
+        <v>0.70526798290059278</v>
+      </c>
+      <c r="J19" s="18">
+        <f t="shared" si="0"/>
+        <v>53.346466592036222</v>
+      </c>
+      <c r="K19" s="18">
+        <f t="shared" si="0"/>
+        <v>60.987695146146315</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="18">
+        <f t="shared" ref="C20:K20" si="1">C6*100</f>
+        <v>51.761636804715216</v>
+      </c>
+      <c r="D20" s="18">
+        <f t="shared" si="1"/>
+        <v>55.231838925205409</v>
+      </c>
+      <c r="E20" s="18">
+        <f t="shared" si="1"/>
+        <v>53.033133104407071</v>
+      </c>
+      <c r="F20" s="18">
+        <f t="shared" si="1"/>
+        <v>53.566390550107144</v>
+      </c>
+      <c r="G20" s="18">
+        <f t="shared" si="1"/>
+        <v>57.992648943138192</v>
+      </c>
+      <c r="H20" s="18">
+        <f t="shared" si="1"/>
+        <v>56.151960801123693</v>
+      </c>
+      <c r="I20" s="18">
+        <f t="shared" si="1"/>
+        <v>2.2664482874882692</v>
+      </c>
+      <c r="J20" s="18">
+        <f t="shared" si="1"/>
+        <v>52.0690697840704</v>
+      </c>
+      <c r="K20" s="18">
+        <f t="shared" si="1"/>
+        <v>61.816374686991949</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1">
+        <v>3</v>
+      </c>
+      <c r="C21" s="18">
+        <f t="shared" ref="C21:K21" si="2">C7*100</f>
+        <v>39.691520257217562</v>
+      </c>
+      <c r="D21" s="18">
+        <f t="shared" si="2"/>
+        <v>46.669964652405369</v>
+      </c>
+      <c r="E21" s="18">
+        <f t="shared" si="2"/>
+        <v>36.12456043807672</v>
+      </c>
+      <c r="F21" s="18">
+        <f t="shared" si="2"/>
+        <v>40.560546619190603</v>
+      </c>
+      <c r="G21" s="18">
+        <f t="shared" si="2"/>
+        <v>50.389135708422415</v>
+      </c>
+      <c r="H21" s="18">
+        <f t="shared" si="2"/>
+        <v>50.840258567507369</v>
+      </c>
+      <c r="I21" s="18">
+        <f t="shared" si="2"/>
+        <v>0.1755804008000994</v>
+      </c>
+      <c r="J21" s="18">
+        <f t="shared" si="2"/>
+        <v>24.563242530246409</v>
+      </c>
+      <c r="K21" s="18">
+        <f t="shared" si="2"/>
+        <v>8.2613999455411397E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>4</v>
+      </c>
+      <c r="C22" s="18">
+        <f t="shared" ref="C22:K22" si="3">C8*100</f>
+        <v>39.689351424585773</v>
+      </c>
+      <c r="D22" s="18">
+        <f t="shared" si="3"/>
+        <v>47.746588090129322</v>
+      </c>
+      <c r="E22" s="18">
+        <f t="shared" si="3"/>
+        <v>41.827914800233053</v>
+      </c>
+      <c r="F22" s="18">
+        <f t="shared" si="3"/>
+        <v>46.396150970479077</v>
+      </c>
+      <c r="G22" s="18">
+        <f t="shared" si="3"/>
+        <v>48.609862930973804</v>
+      </c>
+      <c r="H22" s="18">
+        <f t="shared" si="3"/>
+        <v>48.267138745623143</v>
+      </c>
+      <c r="I22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.30990898364572239</v>
+      </c>
+      <c r="J22" s="18">
+        <f t="shared" si="3"/>
+        <v>28.326525691982052</v>
+      </c>
+      <c r="K22" s="18">
+        <f t="shared" si="3"/>
+        <v>0.13761703709420892</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="1">
+        <v>5</v>
+      </c>
+      <c r="C23" s="18">
+        <f t="shared" ref="C23:K23" si="4">C9*100</f>
+        <v>6.7773277906756313</v>
+      </c>
+      <c r="D23" s="18">
+        <f t="shared" si="4"/>
+        <v>62.17732432161133</v>
+      </c>
+      <c r="E23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.14563086768023759</v>
+      </c>
+      <c r="F23" s="18">
+        <f t="shared" si="4"/>
+        <v>62.680609145343112</v>
+      </c>
+      <c r="G23" s="18">
+        <f t="shared" si="4"/>
+        <v>62.963182279656451</v>
+      </c>
+      <c r="H23" s="18">
+        <f t="shared" si="4"/>
+        <v>66.21206499633918</v>
+      </c>
+      <c r="I23" s="18">
+        <f t="shared" si="4"/>
+        <v>2.400622630882417E-2</v>
+      </c>
+      <c r="J23" s="18">
+        <f t="shared" si="4"/>
+        <v>0.28604909222318831</v>
+      </c>
+      <c r="K23" s="18">
+        <f t="shared" si="4"/>
+        <v>60.935182980998825</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="1">
+        <v>6</v>
+      </c>
+      <c r="C24" s="18">
+        <f t="shared" ref="C24:K24" si="5">C10*100</f>
+        <v>29.36580585396726</v>
+      </c>
+      <c r="D24" s="18">
+        <f t="shared" si="5"/>
+        <v>37.882610243073472</v>
+      </c>
+      <c r="E24" s="18">
+        <f t="shared" si="5"/>
+        <v>2.3259038975479589</v>
+      </c>
+      <c r="F24" s="18">
+        <f t="shared" si="5"/>
+        <v>37.545524986367177</v>
+      </c>
+      <c r="G24" s="18">
+        <f t="shared" si="5"/>
+        <v>39.98186179699897</v>
+      </c>
+      <c r="H24" s="18">
+        <f t="shared" si="5"/>
+        <v>40.673117510599972</v>
+      </c>
+      <c r="I24" s="18">
+        <f t="shared" si="5"/>
+        <v>2.2651044622337281E-2</v>
+      </c>
+      <c r="J24" s="18">
+        <f t="shared" si="5"/>
+        <v>0.29202912180879032</v>
+      </c>
+      <c r="K24" s="18">
+        <f t="shared" si="5"/>
+        <v>1.264620557706511E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="1">
+        <v>7</v>
+      </c>
+      <c r="C25" s="18">
+        <f t="shared" ref="C25:K25" si="6">C11*100</f>
+        <v>15.31095814839823</v>
+      </c>
+      <c r="D25" s="18">
+        <f t="shared" si="6"/>
+        <v>28.31055406058216</v>
+      </c>
+      <c r="E25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.82971293421046544</v>
+      </c>
+      <c r="F25" s="18">
+        <f t="shared" si="6"/>
+        <v>28.379627737243919</v>
+      </c>
+      <c r="G25" s="18">
+        <f t="shared" si="6"/>
+        <v>38.572668657974383</v>
+      </c>
+      <c r="H25" s="18">
+        <f t="shared" si="6"/>
+        <v>40.283661619656677</v>
+      </c>
+      <c r="I25" s="18">
+        <f t="shared" si="6"/>
+        <v>2.37658331154177E-2</v>
+      </c>
+      <c r="J25" s="18">
+        <f t="shared" si="6"/>
+        <v>0.28440836520917051</v>
+      </c>
+      <c r="K25" s="18">
+        <f t="shared" si="6"/>
+        <v>1.331933890226125E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="1">
+        <v>8</v>
+      </c>
+      <c r="C26" s="18">
+        <f t="shared" ref="C26:K26" si="7">C12*100</f>
+        <v>50.303987817960646</v>
+      </c>
+      <c r="D26" s="18">
+        <f t="shared" si="7"/>
+        <v>63.001134459516194</v>
+      </c>
+      <c r="E26" s="18">
+        <f t="shared" si="7"/>
+        <v>57.892342770524074</v>
+      </c>
+      <c r="F26" s="18">
+        <f t="shared" si="7"/>
+        <v>56.869526640991111</v>
+      </c>
+      <c r="G26" s="18">
+        <f t="shared" si="7"/>
+        <v>62.83844572608136</v>
+      </c>
+      <c r="H26" s="18">
+        <f t="shared" si="7"/>
+        <v>62.786695340922662</v>
+      </c>
+      <c r="I26" s="18">
+        <f t="shared" si="7"/>
+        <v>3.9183696341225844</v>
+      </c>
+      <c r="J26" s="18">
+        <f t="shared" si="7"/>
+        <v>55.209161250567853</v>
+      </c>
+      <c r="K26" s="18">
+        <f t="shared" si="7"/>
+        <v>61.260249678497061</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B16:K16"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:K12">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19:K26">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color theme="0"/>
+        <color theme="3" tint="0.39997558519241921"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -8811,18 +10436,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="B2" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -9150,18 +10775,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -9489,18 +11114,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="B2" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -9819,6 +11444,684 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:K12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="11" width="12.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="30"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="2"/>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>3.594244980400001</v>
+      </c>
+      <c r="D5" s="5">
+        <v>3.6157147749999998</v>
+      </c>
+      <c r="E5" s="5">
+        <v>3.3854246967999999</v>
+      </c>
+      <c r="F5" s="5">
+        <v>3.7316625503999998</v>
+      </c>
+      <c r="G5" s="5">
+        <v>3.6852943248000001</v>
+      </c>
+      <c r="H5" s="5">
+        <v>3.8447531287999999</v>
+      </c>
+      <c r="I5" s="5">
+        <v>3.0772555918000002</v>
+      </c>
+      <c r="J5" s="5">
+        <v>3.3651249924000002</v>
+      </c>
+      <c r="K5" s="5">
+        <v>2.8922452831999999</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="5">
+        <v>3.563196773</v>
+      </c>
+      <c r="D6" s="5">
+        <v>3.5479311776000002</v>
+      </c>
+      <c r="E6" s="5">
+        <v>3.3061578886</v>
+      </c>
+      <c r="F6" s="5">
+        <v>3.5831971519999999</v>
+      </c>
+      <c r="G6" s="5">
+        <v>3.5861631946000001</v>
+      </c>
+      <c r="H6" s="5">
+        <v>3.6144358392</v>
+      </c>
+      <c r="I6" s="5">
+        <v>2.9383141834000002</v>
+      </c>
+      <c r="J6" s="5">
+        <v>3.3028380978</v>
+      </c>
+      <c r="K6" s="5">
+        <v>2.7414397043999998</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="5">
+        <v>3.2911644072000001</v>
+      </c>
+      <c r="D7" s="5">
+        <v>3.2112445254000002</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2.9461782780000001</v>
+      </c>
+      <c r="F7" s="5">
+        <v>3.3699958329999999</v>
+      </c>
+      <c r="G7" s="5">
+        <v>3.2886881697999999</v>
+      </c>
+      <c r="H7" s="5">
+        <v>3.4532627169999999</v>
+      </c>
+      <c r="I7" s="5">
+        <v>2.6335465033999998</v>
+      </c>
+      <c r="J7" s="5">
+        <v>2.9524096886</v>
+      </c>
+      <c r="K7" s="5">
+        <v>2.4297331174000001</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5">
+        <v>3.4624601702</v>
+      </c>
+      <c r="D8" s="5">
+        <v>3.2543473829999998</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2.9993493536</v>
+      </c>
+      <c r="F8" s="5">
+        <v>3.468800426400001</v>
+      </c>
+      <c r="G8" s="5">
+        <v>3.3346482244</v>
+      </c>
+      <c r="H8" s="5">
+        <v>3.5576184359999998</v>
+      </c>
+      <c r="I8" s="5">
+        <v>2.637737059</v>
+      </c>
+      <c r="J8" s="5">
+        <v>3.0517040872000001</v>
+      </c>
+      <c r="K8" s="5">
+        <v>2.4335699248</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>5</v>
+      </c>
+      <c r="C9" s="5">
+        <v>3.2382654456000002</v>
+      </c>
+      <c r="D9" s="5">
+        <v>3.3154641873999999</v>
+      </c>
+      <c r="E9" s="5">
+        <v>3.0936368546000002</v>
+      </c>
+      <c r="F9" s="5">
+        <v>3.3800368395999998</v>
+      </c>
+      <c r="G9" s="5">
+        <v>3.3951663779999999</v>
+      </c>
+      <c r="H9" s="5">
+        <v>3.5078487853999998</v>
+      </c>
+      <c r="I9" s="5">
+        <v>2.806311682</v>
+      </c>
+      <c r="J9" s="5">
+        <v>3.0557041630000001</v>
+      </c>
+      <c r="K9" s="5">
+        <v>2.6174101431999999</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <v>6</v>
+      </c>
+      <c r="C10" s="5">
+        <v>3.0756501192000001</v>
+      </c>
+      <c r="D10" s="5">
+        <v>3.1625905421999998</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2.9471850998</v>
+      </c>
+      <c r="F10" s="5">
+        <v>3.2082784827999999</v>
+      </c>
+      <c r="G10" s="5">
+        <v>3.2390817876</v>
+      </c>
+      <c r="H10" s="5">
+        <v>3.3187567668</v>
+      </c>
+      <c r="I10" s="5">
+        <v>2.6622545303999998</v>
+      </c>
+      <c r="J10" s="5">
+        <v>2.9090619283999999</v>
+      </c>
+      <c r="K10" s="5">
+        <v>2.4754210579999998</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>7</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2.8303121367999999</v>
+      </c>
+      <c r="D11" s="5">
+        <v>2.9551308286000002</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2.7349361798</v>
+      </c>
+      <c r="F11" s="5">
+        <v>2.9696072934000002</v>
+      </c>
+      <c r="G11" s="5">
+        <v>3.0223157752000001</v>
+      </c>
+      <c r="H11" s="5">
+        <v>3.1080861080000002</v>
+      </c>
+      <c r="I11" s="5">
+        <v>2.4379237487999998</v>
+      </c>
+      <c r="J11" s="5">
+        <v>2.6695199742</v>
+      </c>
+      <c r="K11" s="5">
+        <v>2.2504644142000001</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>8</v>
+      </c>
+      <c r="C12" s="5">
+        <v>3.7999359529999999</v>
+      </c>
+      <c r="D12" s="5">
+        <v>3.7128866843999999</v>
+      </c>
+      <c r="E12" s="5">
+        <v>3.4575349067999999</v>
+      </c>
+      <c r="F12" s="5">
+        <v>3.8328073242</v>
+      </c>
+      <c r="G12" s="5">
+        <v>3.7685884202</v>
+      </c>
+      <c r="H12" s="5">
+        <v>3.9269315568000001</v>
+      </c>
+      <c r="I12" s="5">
+        <v>3.1755703799999999</v>
+      </c>
+      <c r="J12" s="5">
+        <v>3.4872225442000002</v>
+      </c>
+      <c r="K12" s="5">
+        <v>3.054615707</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:K2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:K12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:K12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="11" width="12.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="33"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="2"/>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>3.1870808022000001</v>
+      </c>
+      <c r="D5" s="5">
+        <v>3.1322498311999998</v>
+      </c>
+      <c r="E5" s="5">
+        <v>3.1664001382000002</v>
+      </c>
+      <c r="F5" s="5">
+        <v>3.195706816</v>
+      </c>
+      <c r="G5" s="5">
+        <v>3.1257463066</v>
+      </c>
+      <c r="H5" s="5">
+        <v>3.1669443662000001</v>
+      </c>
+      <c r="I5" s="5">
+        <v>3.0622621103999998</v>
+      </c>
+      <c r="J5" s="5">
+        <v>3.0859632397999999</v>
+      </c>
+      <c r="K5" s="5">
+        <v>2.5738719032000001</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2.9426952188</v>
+      </c>
+      <c r="D6" s="5">
+        <v>2.9256880937999998</v>
+      </c>
+      <c r="E6" s="5">
+        <v>2.9284908679999999</v>
+      </c>
+      <c r="F6" s="5">
+        <v>2.9341236278</v>
+      </c>
+      <c r="G6" s="5">
+        <v>2.9267765498</v>
+      </c>
+      <c r="H6" s="5">
+        <v>2.9314841220000001</v>
+      </c>
+      <c r="I6" s="5">
+        <v>2.9082183750000001</v>
+      </c>
+      <c r="J6" s="5">
+        <v>2.9028577292</v>
+      </c>
+      <c r="K6" s="5">
+        <v>2.5744433426</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2.8925718200000001</v>
+      </c>
+      <c r="D7" s="5">
+        <v>2.9423958934000001</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2.9015243705999998</v>
+      </c>
+      <c r="F7" s="5">
+        <v>2.9558383250000002</v>
+      </c>
+      <c r="G7" s="5">
+        <v>2.9571444722</v>
+      </c>
+      <c r="H7" s="5">
+        <v>2.9980432064000002</v>
+      </c>
+      <c r="I7" s="5">
+        <v>2.6290294109999999</v>
+      </c>
+      <c r="J7" s="5">
+        <v>2.8257950444</v>
+      </c>
+      <c r="K7" s="5">
+        <v>2.4289984096000001</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5">
+        <v>2.9153205504000002</v>
+      </c>
+      <c r="D8" s="5">
+        <v>2.9262051104000002</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2.9120279710000001</v>
+      </c>
+      <c r="F8" s="5">
+        <v>2.9494708574000001</v>
+      </c>
+      <c r="G8" s="5">
+        <v>2.9321371956000002</v>
+      </c>
+      <c r="H8" s="5">
+        <v>2.971348823</v>
+      </c>
+      <c r="I8" s="5">
+        <v>2.6287028742</v>
+      </c>
+      <c r="J8" s="5">
+        <v>2.8662039734000002</v>
+      </c>
+      <c r="K8" s="5">
+        <v>2.4320460864000002</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>5</v>
+      </c>
+      <c r="C9" s="5">
+        <v>3.1998701602000001</v>
+      </c>
+      <c r="D9" s="5">
+        <v>3.1527400154</v>
+      </c>
+      <c r="E9" s="5">
+        <v>3.0929293582000001</v>
+      </c>
+      <c r="F9" s="5">
+        <v>3.2304013509999998</v>
+      </c>
+      <c r="G9" s="5">
+        <v>3.1416377642</v>
+      </c>
+      <c r="H9" s="5">
+        <v>3.1835161088000001</v>
+      </c>
+      <c r="I9" s="5">
+        <v>2.8062572592000001</v>
+      </c>
+      <c r="J9" s="5">
+        <v>3.0551327235999999</v>
+      </c>
+      <c r="K9" s="5">
+        <v>2.5741440172000001</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <v>6</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2.9744781339999999</v>
+      </c>
+      <c r="D10" s="5">
+        <v>3.0218803928</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2.9447904966</v>
+      </c>
+      <c r="F10" s="5">
+        <v>3.0207647253999999</v>
+      </c>
+      <c r="G10" s="5">
+        <v>3.0272682500000001</v>
+      </c>
+      <c r="H10" s="5">
+        <v>3.0335540833999999</v>
+      </c>
+      <c r="I10" s="5">
+        <v>2.6622273189999999</v>
+      </c>
+      <c r="J10" s="5">
+        <v>2.9084088548000002</v>
+      </c>
+      <c r="K10" s="5">
+        <v>2.4753938465999998</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>7</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2.7683789904</v>
+      </c>
+      <c r="D11" s="5">
+        <v>2.9011706224</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2.7334123413999998</v>
+      </c>
+      <c r="F11" s="5">
+        <v>2.8631290852000002</v>
+      </c>
+      <c r="G11" s="5">
+        <v>2.9306677799999998</v>
+      </c>
+      <c r="H11" s="5">
+        <v>2.9337970910000002</v>
+      </c>
+      <c r="I11" s="5">
+        <v>2.4378965373999999</v>
+      </c>
+      <c r="J11" s="5">
+        <v>2.6691934374000001</v>
+      </c>
+      <c r="K11" s="5">
+        <v>2.2504644142000001</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>8</v>
+      </c>
+      <c r="C12" s="5">
+        <v>3.1289300403999998</v>
+      </c>
+      <c r="D12" s="5">
+        <v>3.0807114395999999</v>
+      </c>
+      <c r="E12" s="5">
+        <v>3.0974464506000001</v>
+      </c>
+      <c r="F12" s="5">
+        <v>3.1216645966000001</v>
+      </c>
+      <c r="G12" s="5">
+        <v>3.0804937483999999</v>
+      </c>
+      <c r="H12" s="5">
+        <v>3.1197325872000001</v>
+      </c>
+      <c r="I12" s="5">
+        <v>3.1262361117999999</v>
+      </c>
+      <c r="J12" s="5">
+        <v>3.0428059593999999</v>
+      </c>
+      <c r="K12" s="5">
+        <v>2.5741168058000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:K2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:K12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:K12"/>
@@ -9828,18 +12131,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -10167,18 +12470,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -10506,18 +12809,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -10845,18 +13148,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -11184,18 +13487,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -11523,18 +13826,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>

</xml_diff>